<commit_message>
Extent Report Data driven
</commit_message>
<xml_diff>
--- a/test-data/FormData.xlsx
+++ b/test-data/FormData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2464428\IdeaProjects\Identify_Courses_Coursera\test-data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cognizantonline-my.sharepoint.com/personal/2445477_cognizant_com/Documents/Documents/TrainingDocs/Automation&amp;Selenium/HackthonProjects/Cohort19/Identify Courses_Coursera/Coursera/test-data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE2CAE34-3547-4B53-9541-02A499F06C05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{FE2CAE34-3547-4B53-9541-02A499F06C05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0BE4DB1B-C177-45D8-BD23-6384A50941C5}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="11370" activeTab="1" xr2:uid="{EFFCDA33-2838-4B1C-BBBA-3C118CC4D4C3}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{EFFCDA33-2838-4B1C-BBBA-3C118CC4D4C3}"/>
   </bookViews>
   <sheets>
     <sheet name="ValidData" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="22">
   <si>
     <t>firstName</t>
   </si>
@@ -72,15 +72,6 @@
     <t>company</t>
   </si>
   <si>
-    <t>Krishna</t>
-  </si>
-  <si>
-    <t>Sai</t>
-  </si>
-  <si>
-    <t>kri@cognizant.com</t>
-  </si>
-  <si>
     <t>SDE</t>
   </si>
   <si>
@@ -100,6 +91,18 @@
   </si>
   <si>
     <t>khan</t>
+  </si>
+  <si>
+    <t>Mouneshwar</t>
+  </si>
+  <si>
+    <t>Panchal</t>
+  </si>
+  <si>
+    <t>mounesh@cognizant.com</t>
+  </si>
+  <si>
+    <t>Karnataka</t>
   </si>
 </sst>
 </file>
@@ -494,6 +497,7 @@
   <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
     <col min="3" max="3" width="16.453125" customWidth="1"/>
     <col min="4" max="4" width="10.81640625" bestFit="1" customWidth="1"/>
   </cols>
@@ -535,13 +539,13 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D2">
         <v>1234567890</v>
@@ -550,7 +554,7 @@
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G2">
         <v>1</v>
@@ -559,13 +563,13 @@
         <v>2</v>
       </c>
       <c r="I2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="J2" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="K2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -625,13 +629,13 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D2">
         <v>9876543210</v>
@@ -640,7 +644,7 @@
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G2">
         <v>1</v>
@@ -649,13 +653,13 @@
         <v>2</v>
       </c>
       <c r="I2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="J2" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="K2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>